<commit_message>
Regenerated the Excel index manifest summary.
</commit_message>
<xml_diff>
--- a/pipeline/1_index_construction/indices_manifest.xlsx
+++ b/pipeline/1_index_construction/indices_manifest.xlsx
@@ -540,11 +540,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -629,7 +629,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>E:\\OneDrive\\Studia\\Studia magisterskie\\Masterarbeit 2 - Sozialwissenschaften\\data\\Sat_data_curated</t>
+          <t>CONFIG:sat_data_curated</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>E:\\OneDrive\\Studia\\Studia magisterskie\\Masterarbeit 2 - Sozialwissenschaften\\data\\vector\\freguesia.gpkg</t>
+          <t>CONFIG:repo_data_dir/parishes.geojson</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>freguesia_id</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>E:\\OneDrive\\Studia\\Studia magisterskie\\Masterarbeit 2 - Sozialwissenschaften\\data\\outputs\\indices</t>
+          <t>CONFIG:outputs_indices_dir</t>
         </is>
       </c>
     </row>
@@ -772,17 +772,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>global_defaults</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>age_bins</t>
+          <t>fractional_allocation_threshold_m</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>{"pre_1975": {"codes": [1], "mid_year": 1965, "exclude": false}, "1975_1985": {"codes": [2], "mid_year": 1980, "exclude": false}, "1985_1995": {"codes": [3], "mid_year": 1990, "exclude": false}, "1995_2005": {"codes": [4], "mid_year": 2000, "exclude": false}, "2005_2015": {"codes": [5], "mid_year": 2010, "exclude": false}, "2015_2020": {"codes": [6], "mid_year": null, "exclude": true}}</t>
+          <t>400</t>
         </is>
       </c>
     </row>
@@ -794,10 +794,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>age_bins</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>{"pre_1975": {"codes": [1], "mid_year": 1965, "exclude": false}, "1975_1985": {"codes": [2], "mid_year": 1980, "exclude": false}, "1985_1995": {"codes": [3], "mid_year": 1990, "exclude": false}, "1995_2005": {"codes": [4], "mid_year": 2000, "exclude": false}, "2005_2015": {"codes": [5], "mid_year": 2010, "exclude": false}, "2015_2020": {"codes": [6], "mid_year": null, "exclude": true}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>helpers</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>functions_required_in_runner</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>["recode_age_midyear(age_class, age_bins)", "is_age_bin(age_class, bin_name, age_bins)"]</t>
         </is>
@@ -1190,7 +1207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1199,7 +1216,7 @@
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="29" customWidth="1" min="6" max="6"/>
-    <col width="57" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="49" customWidth="1" min="10" max="10"/>
@@ -1465,7 +1482,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>res_volume &gt; 0 &amp;&amp; pop &gt; 0</t>
+          <t>(res_volume &gt; 0) &amp;&amp; (pop &gt; 0)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1520,7 +1537,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>res_volume &gt; 0 &amp;&amp; pop &gt; 0</t>
+          <t>(res_volume &gt; 0) &amp;&amp; (pop &gt; 0)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1571,7 +1588,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>res_volume &gt; 0 &amp;&amp; mid_year != null</t>
+          <t>(res_volume &gt; 0) &amp;&amp; (mid_year != null)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1944,7 +1961,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>res_area &gt; 0 &amp;&amp; pop &gt; 0</t>
+          <t>(res_area &gt; 0) &amp;&amp; (pop &gt; 0)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1995,7 +2012,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>pop &gt; 0 &amp;&amp; res_area &gt; 0</t>
+          <t>(pop &gt; 0) &amp;&amp; (res_area &gt; 0)</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2050,7 +2067,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>pop &gt; 0 &amp;&amp; res_area &gt; 0</t>
+          <t>(pop &gt; 0) &amp;&amp; (res_area &gt; 0)</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2101,7 +2118,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>res_volume &gt; 0 &amp;&amp; mid_year != null</t>
+          <t>(res_volume &gt; 0) &amp;&amp; (mid_year != null)</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2152,7 +2169,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>res_volume &gt; 0 &amp;&amp; mid_year != null</t>
+          <t>(res_volume &gt; 0) &amp;&amp; (mid_year != null)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2203,7 +2220,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>res_volume &gt; 0 &amp;&amp; mid_year != null</t>
+          <t>(res_volume &gt; 0) &amp;&amp; (mid_year != null)</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2254,7 +2271,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>res_volume &gt; 0 &amp;&amp; (res_area + nres_area) &gt; 0</t>
+          <t>(res_volume &gt; 0) &amp;&amp; ((res_area + nres_area) &gt; 0)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2279,7 +2296,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita</t>
+          <t>ntl</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2289,52 +2306,44 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>(ntl*res_share*pop)/res_volume as ratio of sums.</t>
+          <t>Total residential-attributed night-time light: sum(ntl_intensity * residential built-up share).</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>["NTL", "Surface", "Surface_NRES", "Population", "Volume"]</t>
+          <t>["NTL", "Surface", "Surface_NRES"]</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>{"ntl": "NTL", "res_area": "Surface", "nres_area": "Surface_NRES", "pop": "Population", "res_volume": "Volume"}</t>
+          <t>{"ntl": "NTL", "res_area": "Surface", "nres_area": "Surface_NRES"}</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>proxy</t>
+          <t>ntl_res</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>res_volume &gt; 0 &amp;&amp; pop &gt; 0 &amp;&amp; (res_area + nres_area) &gt; 0</t>
+          <t>((res_area + nres_area) &gt; 0)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>ratio_of_sums</t>
+          <t>sum</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>ntl * (res_area / (res_area + nres_area)) * pop</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>res_volume</t>
-        </is>
-      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ntl_per_res_vol_distrib</t>
+          <t>ntl_per_capita</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2344,48 +2353,52 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Distribution of ntl_per_res_vol across cells weighted by res_volume.</t>
+          <t>Residential-attributed night-time light per capita: sum(ntl_intensity * residential built-up share) / sum(population).</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>["NTL", "Surface", "Surface_NRES", "Volume"]</t>
+          <t>["NTL", "Surface", "Surface_NRES", "Population"]</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>{"ntl": "NTL", "res_area": "Surface", "nres_area": "Surface_NRES", "res_volume": "Volume"}</t>
+          <t>{"ntl": "NTL", "res_area": "Surface", "nres_area": "Surface_NRES", "pop": "Population"}</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>ntl_res / pop</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>res_volume &gt; 0 &amp;&amp; (res_area + nres_area) &gt; 0</t>
+          <t>(pop &gt; 0) &amp;&amp; ((res_area + nres_area) &gt; 0)</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>weighted_distribution</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>res_volume</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+          <t>ratio_of_sums</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>ntl * (res_area / (res_area + nres_area))</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>pop</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita_distrib</t>
+          <t>energy_per_vol_per_capita</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2395,7 +2408,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Distribution of (ntl*res_share*pop)/res_volume across cells, weighted by population.</t>
+          <t>(ntl*res_share*pop)/res_volume as ratio of sums.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2410,73 +2423,77 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>proxy</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>res_volume &gt; 0 &amp;&amp; pop &gt; 0 &amp;&amp; (res_area + nres_area) &gt; 0</t>
+          <t>(res_volume &gt; 0) &amp;&amp; (pop &gt; 0) &amp;&amp; ((res_area + nres_area) &gt; 0)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>weighted_distribution</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>pop</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+          <t>ratio_of_sums</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>ntl * (res_area / (res_area + nres_area)) * pop</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>res_volume</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>delta_pm_25</t>
+          <t>ntl_per_res_vol_distrib</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Heating by combustion</t>
+          <t>Energy consumption proxies</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PM2.5 delta (heating season vs rest of year), population-weighted.</t>
+          <t>Distribution of ntl_per_res_vol across cells weighted by res_volume.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>["PM_2_5_delta", "Population"]</t>
+          <t>["NTL", "Surface", "Surface_NRES", "Volume"]</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>{"delta": "PM_2_5_delta", "pop": "Population"}</t>
+          <t>{"ntl": "NTL", "res_area": "Surface", "nres_area": "Surface_NRES", "res_volume": "Volume"}</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>delta</t>
+          <t>val</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>pop &gt; 0</t>
+          <t>(res_volume &gt; 0) &amp;&amp; ((res_area + nres_area) &gt; 0)</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>weighted_mean</t>
+          <t>weighted_distribution</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>pop</t>
+          <t>res_volume</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -2487,42 +2504,42 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>standard_delta_pm_25</t>
+          <t>energy_per_vol_per_capita_distrib</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Heating by combustion</t>
+          <t>Energy consumption proxies</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PM2.5 delta standardized by average PM2.5, population-weighted.</t>
+          <t>Distribution of (ntl*res_share*pop)/res_volume across cells, weighted by population.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>["PM_2_5_delta", "PM_2_5_average", "Population"]</t>
+          <t>["NTL", "Surface", "Surface_NRES", "Population", "Volume"]</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>{"delta": "PM_2_5_delta", "avg": "PM_2_5_average", "pop": "Population"}</t>
+          <t>{"ntl": "NTL", "res_area": "Surface", "nres_area": "Surface_NRES", "pop": "Population", "res_volume": "Volume"}</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>std_delta</t>
+          <t>val</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>pop &gt; 0 &amp;&amp; avg &gt; 0</t>
+          <t>(res_volume &gt; 0) &amp;&amp; (pop &gt; 0) &amp;&amp; ((res_area + nres_area) &gt; 0)</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>weighted_mean</t>
+          <t>weighted_distribution</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2538,7 +2555,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>delta_pm_25_per_capita</t>
+          <t>delta_pm_25</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2548,7 +2565,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Cell-level delta_pm25/population, averaged across populated cells.</t>
+          <t>PM2.5 delta (heating season vs rest of year), population-weighted.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2563,7 +2580,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>delta</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2573,10 +2590,14 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr"/>
+          <t>weighted_mean</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>pop</t>
+        </is>
+      </c>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
@@ -2585,7 +2606,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>delta_bc</t>
+          <t>standard_delta_pm_25</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2595,27 +2616,27 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Black carbon delta, population-weighted.</t>
+          <t>PM2.5 delta standardized by average PM2.5, population-weighted.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>["BC_delta", "Population"]</t>
+          <t>["PM_2_5_delta", "PM_2_5_average", "Population"]</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>{"delta": "BC_delta", "pop": "Population"}</t>
+          <t>{"delta": "PM_2_5_delta", "avg": "PM_2_5_average", "pop": "Population"}</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>delta</t>
+          <t>std_delta</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>pop &gt; 0</t>
+          <t>(pop &gt; 0) &amp;&amp; (avg &gt; 0)</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2636,7 +2657,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>standard_delta_bc</t>
+          <t>delta_pm_25_per_capita</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2646,39 +2667,35 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>BC delta standardized by average BC, population-weighted.</t>
+          <t>Cell-level delta_pm25/population, averaged across populated cells.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>["BC_delta", "BC_average", "Population"]</t>
+          <t>["PM_2_5_delta", "Population"]</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>{"delta": "BC_delta", "avg": "BC_average", "pop": "Population"}</t>
+          <t>{"delta": "PM_2_5_delta", "pop": "Population"}</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>std_delta</t>
+          <t>val</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>pop &gt; 0 &amp;&amp; avg &gt; 0</t>
+          <t>pop &gt; 0</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>weighted_mean</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>pop</t>
-        </is>
-      </c>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
@@ -2687,7 +2704,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>delta_bc_per_capita</t>
+          <t>delta_bc</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2697,7 +2714,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Cell-level BC_delta/population, averaged across populated cells.</t>
+          <t>Black carbon delta, population-weighted.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2712,7 +2729,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>delta</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2722,10 +2739,14 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr"/>
+          <t>weighted_mean</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>pop</t>
+        </is>
+      </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
@@ -2734,7 +2755,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>delta_oc</t>
+          <t>standard_delta_bc</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2744,27 +2765,27 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Organic carbon delta, population-weighted.</t>
+          <t>BC delta standardized by average BC, population-weighted.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>["OC_delta", "Population"]</t>
+          <t>["BC_delta", "BC_average", "Population"]</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>{"delta": "OC_delta", "pop": "Population"}</t>
+          <t>{"delta": "BC_delta", "avg": "BC_average", "pop": "Population"}</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>delta</t>
+          <t>std_delta</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>pop &gt; 0</t>
+          <t>(pop &gt; 0) &amp;&amp; (avg &gt; 0)</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2785,7 +2806,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>standard_delta_oc</t>
+          <t>delta_bc_per_capita</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2795,39 +2816,35 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>OC delta standardized by average OC, population-weighted.</t>
+          <t>Cell-level BC_delta/population, averaged across populated cells.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>["OC_delta", "OC_average", "Population"]</t>
+          <t>["BC_delta", "Population"]</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>{"delta": "OC_delta", "avg": "OC_average", "pop": "Population"}</t>
+          <t>{"delta": "BC_delta", "pop": "Population"}</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>std_delta</t>
+          <t>val</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>pop &gt; 0 &amp;&amp; avg &gt; 0</t>
+          <t>pop &gt; 0</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>weighted_mean</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>pop</t>
-        </is>
-      </c>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
@@ -2836,7 +2853,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>delta_oc_per_capita</t>
+          <t>delta_oc</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2846,7 +2863,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Cell-level OC_delta/population, averaged across populated cells.</t>
+          <t>Organic carbon delta, population-weighted.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2861,7 +2878,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>delta</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2871,10 +2888,14 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr"/>
+          <t>weighted_mean</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>pop</t>
+        </is>
+      </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
@@ -2883,37 +2904,37 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>hdd_18</t>
+          <t>standard_delta_oc</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Need/heat exposure</t>
+          <t>Heating by combustion</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Heating Degree Days below 18°C, population-weighted.</t>
+          <t>OC delta standardized by average OC, population-weighted.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>["ERA5-Land_HDD", "Population"]</t>
+          <t>["OC_delta", "OC_average", "Population"]</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>{"hdd": "ERA5-Land_HDD", "pop": "Population"}</t>
+          <t>{"delta": "OC_delta", "avg": "OC_average", "pop": "Population"}</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>hdd</t>
+          <t>std_delta</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>pop &gt;= 0</t>
+          <t>(pop &gt; 0) &amp;&amp; (avg &gt; 0)</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2934,49 +2955,45 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>cdd_25</t>
+          <t>delta_oc_per_capita</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Need/heat exposure</t>
+          <t>Heating by combustion</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Cooling Degree Days above 25°C, population-weighted.</t>
+          <t>Cell-level OC_delta/population, averaged across populated cells.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>["ERA5-Land_CDD", "Population"]</t>
+          <t>["OC_delta", "Population"]</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>{"cdd": "ERA5-Land_CDD", "pop": "Population"}</t>
+          <t>{"delta": "OC_delta", "pop": "Population"}</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>cdd</t>
+          <t>val</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>pop &gt;= 0</t>
+          <t>pop &gt; 0</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>weighted_mean</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>pop</t>
-        </is>
-      </c>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
@@ -2985,7 +3002,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>extreme_heat</t>
+          <t>hdd_18</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2995,22 +3012,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Average temperature for 6th–10th hottest days, population-weighted.</t>
+          <t>Heating Degree Days below 18°C, population-weighted.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>["ERA5-Land_extreme_heat", "Population"]</t>
+          <t>["ERA5-Land_HDD", "Population"]</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>{"heat": "ERA5-Land_extreme_heat", "pop": "Population"}</t>
+          <t>{"hdd": "ERA5-Land_HDD", "pop": "Population"}</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>heat</t>
+          <t>hdd</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3036,7 +3053,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>extreme_cold</t>
+          <t>cdd_25</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3046,22 +3063,22 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Average temperature for 6th–10th coldest days, population-weighted.</t>
+          <t>Cooling Degree Days above 25°C, population-weighted.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>["ERA5-Land_extreme_cold", "Population"]</t>
+          <t>["ERA5-Land_CDD", "Population"]</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>{"cold": "ERA5-Land_extreme_cold", "pop": "Population"}</t>
+          <t>{"cdd": "ERA5-Land_CDD", "pop": "Population"}</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>cdd</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3083,6 +3100,108 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>extreme_heat</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Need/heat exposure</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Average temperature for 6th–10th hottest days, population-weighted.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>["ERA5-Land_extreme_heat", "Population"]</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>{"heat": "ERA5-Land_extreme_heat", "pop": "Population"}</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>heat</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>pop &gt;= 0</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>weighted_mean</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>pop</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>extreme_cold</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Need/heat exposure</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Average temperature for 6th–10th coldest days, population-weighted.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>["ERA5-Land_extreme_cold", "Population"]</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>{"cold": "ERA5-Land_extreme_cold", "pop": "Population"}</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>cold</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>pop &gt;= 0</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>weighted_mean</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>pop</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3095,7 +3214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3514,7 +3633,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita</t>
+          <t>ntl</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3531,24 +3650,24 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita</t>
+          <t>ntl</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>proxy</t>
+          <t>ntl_res</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>(ntl * res_share * pop) / res_volume</t>
+          <t>ntl * res_share</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ntl_per_res_vol_distrib</t>
+          <t>ntl_per_capita</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3565,24 +3684,24 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ntl_per_res_vol_distrib</t>
+          <t>ntl_per_capita</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>ntl_res</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>(ntl * res_share) / res_volume</t>
+          <t>ntl * res_share</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita_distrib</t>
+          <t>energy_per_vol_per_capita</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3599,12 +3718,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita_distrib</t>
+          <t>energy_per_vol_per_capita</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>proxy</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3616,24 +3735,24 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>standard_delta_pm_25</t>
+          <t>ntl_per_res_vol_distrib</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>std_delta</t>
+          <t>res_share</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>delta / avg</t>
+          <t>res_area / (res_area + nres_area)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>delta_pm_25_per_capita</t>
+          <t>ntl_per_res_vol_distrib</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3643,31 +3762,31 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>delta / pop</t>
+          <t>(ntl * res_share) / res_volume</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>standard_delta_bc</t>
+          <t>energy_per_vol_per_capita_distrib</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>std_delta</t>
+          <t>res_share</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>delta / avg</t>
+          <t>res_area / (res_area + nres_area)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>delta_bc_per_capita</t>
+          <t>energy_per_vol_per_capita_distrib</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3677,14 +3796,14 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>delta / pop</t>
+          <t>(ntl * res_share * pop) / res_volume</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>standard_delta_oc</t>
+          <t>standard_delta_pm_25</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3701,15 +3820,83 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>delta_pm_25_per_capita</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>val</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>delta / pop</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>standard_delta_bc</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>std_delta</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>delta / avg</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>delta_bc_per_capita</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>val</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>delta / pop</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>standard_delta_oc</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>std_delta</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>delta / avg</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>delta_oc_per_capita</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>val</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>delta / pop</t>
         </is>
@@ -3828,7 +4015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4286,83 +4473,83 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita</t>
+          <t>ntl</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ratio_of_sums</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>ntl * (res_area / (res_area + nres_area)) * pop</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>res_volume</t>
-        </is>
-      </c>
+          <t>sum</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ntl_per_res_vol_distrib</t>
+          <t>ntl_per_capita</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>weighted_distribution</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>res_volume</t>
-        </is>
-      </c>
+          <t>ratio_of_sums</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ntl * (res_area / (res_area + nres_area))</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>pop</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita_distrib</t>
+          <t>energy_per_vol_per_capita</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>weighted_distribution</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>pop</t>
-        </is>
-      </c>
+          <t>ratio_of_sums</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ntl * (res_area / (res_area + nres_area)) * pop</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>res_volume</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>delta_pm_25</t>
+          <t>ntl_per_res_vol_distrib</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>weighted_mean</t>
+          <t>weighted_distribution</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>pop</t>
+          <t>res_volume</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
@@ -4370,12 +4557,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>standard_delta_pm_25</t>
+          <t>energy_per_vol_per_capita_distrib</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>weighted_mean</t>
+          <t>weighted_distribution</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -4390,23 +4577,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>delta_pm_25_per_capita</t>
+          <t>delta_pm_25</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>weighted_mean</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>pop</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>delta_bc</t>
+          <t>standard_delta_pm_25</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4426,43 +4617,43 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>standard_delta_bc</t>
+          <t>delta_pm_25_per_capita</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>weighted_mean</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>pop</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>delta_bc_per_capita</t>
+          <t>delta_bc</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>weighted_mean</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>pop</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>delta_oc</t>
+          <t>standard_delta_bc</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4482,43 +4673,43 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>standard_delta_oc</t>
+          <t>delta_bc_per_capita</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>weighted_mean</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>pop</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>delta_oc_per_capita</t>
+          <t>delta_oc</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>weighted_mean</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>pop</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>hdd_18</t>
+          <t>standard_delta_oc</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4538,27 +4729,23 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>cdd_25</t>
+          <t>delta_oc_per_capita</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>weighted_mean</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>pop</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>extreme_heat</t>
+          <t>hdd_18</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4578,7 +4765,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>extreme_cold</t>
+          <t>cdd_25</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4594,6 +4781,46 @@
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>extreme_heat</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>weighted_mean</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>pop</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>extreme_cold</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>weighted_mean</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>pop</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4984,7 +5211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -5437,51 +5664,51 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita</t>
+          <t>ntl</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita</t>
+          <t>ntl</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ntl*people/m3</t>
+          <t>ntl</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ntl_per_res_vol_distrib</t>
+          <t>ntl_per_capita</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ntl_per_res_vol_p10</t>
+          <t>ntl_per_capita</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ntl/m3</t>
+          <t>ntl/person</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ntl_per_res_vol_distrib</t>
+          <t>energy_per_vol_per_capita</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ntl_per_res_vol_p50</t>
+          <t>energy_per_vol_per_capita</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ntl/m3</t>
+          <t>ntl*people/m3</t>
         </is>
       </c>
     </row>
@@ -5493,7 +5720,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ntl_per_res_vol_p90</t>
+          <t>ntl_per_res_vol_p10</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -5510,46 +5737,46 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ntl_per_res_vol_gini</t>
+          <t>ntl_per_res_vol_p50</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>ntl/m3</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita_distrib</t>
+          <t>ntl_per_res_vol_distrib</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita_p10</t>
+          <t>ntl_per_res_vol_p90</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ntl*people/m3</t>
+          <t>ntl/m3</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita_distrib</t>
+          <t>ntl_per_res_vol_distrib</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita_p50</t>
+          <t>ntl_per_res_vol_gini</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ntl*people/m3</t>
+          <t>index</t>
         </is>
       </c>
     </row>
@@ -5561,7 +5788,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita_p90</t>
+          <t>energy_per_vol_per_capita_p10</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -5578,231 +5805,265 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>energy_per_vol_per_capita_gini</t>
+          <t>energy_per_vol_per_capita_p50</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>ntl*people/m3</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>delta_pm_25</t>
+          <t>energy_per_vol_per_capita_distrib</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>delta_pm_25</t>
+          <t>energy_per_vol_per_capita_p90</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ug/m3</t>
+          <t>ntl*people/m3</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>standard_delta_pm_25</t>
+          <t>energy_per_vol_per_capita_distrib</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>standard_delta_pm_25</t>
+          <t>energy_per_vol_per_capita_gini</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ratio</t>
+          <t>index</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>delta_pm_25_per_capita</t>
+          <t>delta_pm_25</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>delta_pm_25_per_capita</t>
+          <t>delta_pm_25</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ug/m3/person</t>
+          <t>ug/m3</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>delta_bc</t>
+          <t>standard_delta_pm_25</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>delta_bc</t>
+          <t>standard_delta_pm_25</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ug/m3</t>
+          <t>ratio</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>standard_delta_bc</t>
+          <t>delta_pm_25_per_capita</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>standard_delta_bc</t>
+          <t>delta_pm_25_per_capita</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ratio</t>
+          <t>ug/m3/person</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>delta_bc_per_capita</t>
+          <t>delta_bc</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>delta_bc_per_capita</t>
+          <t>delta_bc</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ug/m3/person</t>
+          <t>ug/m3</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>delta_oc</t>
+          <t>standard_delta_bc</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>delta_oc</t>
+          <t>standard_delta_bc</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ug/m3</t>
+          <t>ratio</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>standard_delta_oc</t>
+          <t>delta_bc_per_capita</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>standard_delta_oc</t>
+          <t>delta_bc_per_capita</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ratio</t>
+          <t>ug/m3/person</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>delta_oc_per_capita</t>
+          <t>delta_oc</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>delta_oc_per_capita</t>
+          <t>delta_oc</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ug/m3/person</t>
+          <t>ug/m3</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>hdd_18</t>
+          <t>standard_delta_oc</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>hdd_18</t>
+          <t>standard_delta_oc</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>days</t>
+          <t>ratio</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>cdd_25</t>
+          <t>delta_oc_per_capita</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>cdd_25</t>
+          <t>delta_oc_per_capita</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>days</t>
+          <t>ug/m3/person</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>extreme_heat</t>
+          <t>hdd_18</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>extreme_heat</t>
+          <t>hdd_18</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>days</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>cdd_25</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>cdd_25</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>extreme_heat</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>extreme_heat</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>extreme_cold</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>extreme_cold</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>C</t>
         </is>

</xml_diff>